<commit_message>
Optimized the helper methods in SimulatorWorkflowTests file
</commit_message>
<xml_diff>
--- a/TestProjectArgos/Test data/AutomationConfig.xlsx
+++ b/TestProjectArgos/Test data/AutomationConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3PA_SCHA1\Downloads\VS backup\TestProjectArgos\TestProjectArgos\Test data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB88545D-0E06-486A-9F1B-FEF34BE9AD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B256F7-9F44-4757-B5BA-5153A0694722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
-    <x:workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" firstSheet="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <x:workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" firstSheet="0" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Configuration" sheetId="1" r:id="rId1"/>
@@ -79,13 +79,13 @@
     <x:t>Result</x:t>
   </x:si>
   <x:si>
-    <x:t>argossim19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>p19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>arp19</x:t>
+    <x:t>argossim20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>p20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>arp20</x:t>
   </x:si>
   <x:si>
     <x:t>Male</x:t>
@@ -617,7 +617,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="C2" s="3">
-        <x:v>36206</x:v>
+        <x:v>35841</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>20</x:v>

</xml_diff>